<commit_message>
Actual Test Results + Bug Fixes
</commit_message>
<xml_diff>
--- a/Feature_Testing_Answered.xlsx
+++ b/Feature_Testing_Answered.xlsx
@@ -431,8 +431,8 @@
     <col width="45" customWidth="1" min="5" max="5"/>
     <col width="45" customWidth="1" min="6" max="6"/>
     <col width="45" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -514,17 +514,17 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Dashboard correctly retrieves and displays data charts and summaries.</t>
+          <t>Test execution aborted. System threw SQLSTATE[HY000]: General error: 1 no such table: INFORMATION_SCHEMA.KEY_COLUMN_USAGE.</t>
         </is>
       </c>
       <c r="H2" s="1" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Fail</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>The application uses MySQL-specific raw schema queries (INFORMATION_SCHEMA) which are incompatible with the automated testing environment (SQLite in-memory DB). Tests crash during database migration/initialization.</t>
         </is>
       </c>
     </row>
@@ -561,17 +561,17 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Asset is successfully added to the database and a success message is displayed.</t>
+          <t>Test execution aborted. System threw SQLSTATE[HY000]: General error: 1 no such table: INFORMATION_SCHEMA.KEY_COLUMN_USAGE.</t>
         </is>
       </c>
       <c r="H3" s="1" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Fail</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>The application uses MySQL-specific raw schema queries (INFORMATION_SCHEMA) which are incompatible with the automated testing environment (SQLite in-memory DB). Tests crash during database migration/initialization.</t>
         </is>
       </c>
     </row>
@@ -610,17 +610,17 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Item is saved and appears in the items dropdown for future use.</t>
+          <t>Test execution aborted. System threw SQLSTATE[HY000]: General error: 1 no such table: INFORMATION_SCHEMA.KEY_COLUMN_USAGE.</t>
         </is>
       </c>
       <c r="H4" s="1" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Fail</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>The application uses MySQL-specific raw schema queries (INFORMATION_SCHEMA) which are incompatible with the automated testing environment (SQLite in-memory DB). Tests crash during database migration/initialization.</t>
         </is>
       </c>
     </row>
@@ -657,17 +657,17 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Assets matching the filters are displayed. Clicking an asset opens its detailed profile.</t>
+          <t>Test execution aborted. System threw SQLSTATE[HY000]: General error: 1 no such table: INFORMATION_SCHEMA.KEY_COLUMN_USAGE.</t>
         </is>
       </c>
       <c r="H5" s="1" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Fail</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>The application uses MySQL-specific raw schema queries (INFORMATION_SCHEMA) which are incompatible with the automated testing environment (SQLite in-memory DB). Tests crash during database migration/initialization.</t>
         </is>
       </c>
     </row>
@@ -704,17 +704,17 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Asset is successfully transferred. History log is updated with the transfer details.</t>
+          <t>Test execution aborted. System threw SQLSTATE[HY000]: General error: 1 no such table: INFORMATION_SCHEMA.KEY_COLUMN_USAGE.</t>
         </is>
       </c>
       <c r="H6" s="1" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Fail</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>The application uses MySQL-specific raw schema queries (INFORMATION_SCHEMA) which are incompatible with the automated testing environment (SQLite in-memory DB). Tests crash during database migration/initialization.</t>
         </is>
       </c>
     </row>
@@ -752,17 +752,17 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Files are uploaded, stored, and visible on the asset profile.</t>
+          <t>Test execution aborted. System threw SQLSTATE[HY000]: General error: 1 no such table: INFORMATION_SCHEMA.KEY_COLUMN_USAGE.</t>
         </is>
       </c>
       <c r="H7" s="1" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Fail</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>The application uses MySQL-specific raw schema queries (INFORMATION_SCHEMA) which are incompatible with the automated testing environment (SQLite in-memory DB). Tests crash during database migration/initialization.</t>
         </is>
       </c>
     </row>
@@ -800,17 +800,17 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>An Excel/PDF report is generated with correct data and downloaded to the local machine.</t>
+          <t>Test execution aborted. System threw SQLSTATE[HY000]: General error: 1 no such table: INFORMATION_SCHEMA.KEY_COLUMN_USAGE.</t>
         </is>
       </c>
       <c r="H8" s="1" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Fail</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>The application uses MySQL-specific raw schema queries (INFORMATION_SCHEMA) which are incompatible with the automated testing environment (SQLite in-memory DB). Tests crash during database migration/initialization.</t>
         </is>
       </c>
     </row>
@@ -847,17 +847,17 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>A printable view of QR stickers with correct asset information is displayed.</t>
+          <t>Test execution aborted. System threw SQLSTATE[HY000]: General error: 1 no such table: INFORMATION_SCHEMA.KEY_COLUMN_USAGE.</t>
         </is>
       </c>
       <c r="H9" s="1" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Fail</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>The application uses MySQL-specific raw schema queries (INFORMATION_SCHEMA) which are incompatible with the automated testing environment (SQLite in-memory DB). Tests crash during database migration/initialization.</t>
         </is>
       </c>
     </row>
@@ -895,17 +895,17 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Building records are successfully imported and saved to the database.</t>
+          <t>Test execution aborted. System threw SQLSTATE[HY000]: General error: 1 no such table: INFORMATION_SCHEMA.KEY_COLUMN_USAGE.</t>
         </is>
       </c>
       <c r="H10" s="1" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Fail</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>The application uses MySQL-specific raw schema queries (INFORMATION_SCHEMA) which are incompatible with the automated testing environment (SQLite in-memory DB). Tests crash during database migration/initialization.</t>
         </is>
       </c>
     </row>
@@ -930,8 +930,8 @@
     <col width="45" customWidth="1" min="5" max="5"/>
     <col width="45" customWidth="1" min="6" max="6"/>
     <col width="45" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1015,17 +1015,17 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>User status changes to approved. The user can now log in.</t>
+          <t>Test execution aborted. System threw SQLSTATE[HY000]: General error: 1 no such table: INFORMATION_SCHEMA.KEY_COLUMN_USAGE.</t>
         </is>
       </c>
       <c r="H2" s="1" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Fail</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>The application uses MySQL-specific raw schema queries (INFORMATION_SCHEMA) which are incompatible with the automated testing environment (SQLite in-memory DB). Tests crash during database migration/initialization.</t>
         </is>
       </c>
     </row>
@@ -1063,17 +1063,17 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>User account is permanently deleted from the database.</t>
+          <t>Test execution aborted. System threw SQLSTATE[HY000]: General error: 1 no such table: INFORMATION_SCHEMA.KEY_COLUMN_USAGE.</t>
         </is>
       </c>
       <c r="H3" s="1" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Fail</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>The application uses MySQL-specific raw schema queries (INFORMATION_SCHEMA) which are incompatible with the automated testing environment (SQLite in-memory DB). Tests crash during database migration/initialization.</t>
         </is>
       </c>
     </row>
@@ -1111,17 +1111,17 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>User's role is updated in the database and their access rights change immediately.</t>
+          <t>Test execution aborted. System threw SQLSTATE[HY000]: General error: 1 no such table: INFORMATION_SCHEMA.KEY_COLUMN_USAGE.</t>
         </is>
       </c>
       <c r="H4" s="1" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Fail</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>The application uses MySQL-specific raw schema queries (INFORMATION_SCHEMA) which are incompatible with the automated testing environment (SQLite in-memory DB). Tests crash during database migration/initialization.</t>
         </is>
       </c>
     </row>
@@ -1160,17 +1160,17 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>User access is successfully restricted and restored as expected.</t>
+          <t>Test execution aborted. System threw SQLSTATE[HY000]: General error: 1 no such table: INFORMATION_SCHEMA.KEY_COLUMN_USAGE.</t>
         </is>
       </c>
       <c r="H5" s="1" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Fail</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>The application uses MySQL-specific raw schema queries (INFORMATION_SCHEMA) which are incompatible with the automated testing environment (SQLite in-memory DB). Tests crash during database migration/initialization.</t>
         </is>
       </c>
     </row>
@@ -1208,17 +1208,17 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>The announcement is dispatched to all approved users and appears in their notifications list.</t>
+          <t>Test execution aborted. System threw SQLSTATE[HY000]: General error: 1 no such table: INFORMATION_SCHEMA.KEY_COLUMN_USAGE.</t>
         </is>
       </c>
       <c r="H6" s="1" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Fail</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>The application uses MySQL-specific raw schema queries (INFORMATION_SCHEMA) which are incompatible with the automated testing environment (SQLite in-memory DB). Tests crash during database migration/initialization.</t>
         </is>
       </c>
     </row>
@@ -1256,17 +1256,17 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Employee is successfully added to the system registry.</t>
+          <t>Test execution aborted. System threw SQLSTATE[HY000]: General error: 1 no such table: INFORMATION_SCHEMA.KEY_COLUMN_USAGE.</t>
         </is>
       </c>
       <c r="H7" s="1" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Fail</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>The application uses MySQL-specific raw schema queries (INFORMATION_SCHEMA) which are incompatible with the automated testing environment (SQLite in-memory DB). Tests crash during database migration/initialization.</t>
         </is>
       </c>
     </row>
@@ -1302,17 +1302,17 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>System returns a 403 Forbidden error for all Super Admin restricted routes.</t>
+          <t>Test execution aborted. System threw SQLSTATE[HY000]: General error: 1 no such table: INFORMATION_SCHEMA.KEY_COLUMN_USAGE.</t>
         </is>
       </c>
       <c r="H8" s="1" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Fail</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>The application uses MySQL-specific raw schema queries (INFORMATION_SCHEMA) which are incompatible with the automated testing environment (SQLite in-memory DB). Tests crash during database migration/initialization.</t>
         </is>
       </c>
     </row>
@@ -1337,8 +1337,8 @@
     <col width="45" customWidth="1" min="5" max="5"/>
     <col width="45" customWidth="1" min="6" max="6"/>
     <col width="45" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1425,17 +1425,17 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>User is successfully registered and placed in pending approval state. A notification is sent to Super Admins.</t>
+          <t>Test execution aborted. System threw SQLSTATE[HY000]: General error: 1 no such table: INFORMATION_SCHEMA.KEY_COLUMN_USAGE.</t>
         </is>
       </c>
       <c r="H2" s="1" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Fail</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>The application uses MySQL-specific raw schema queries (INFORMATION_SCHEMA) which are incompatible with the automated testing environment (SQLite in-memory DB). Tests crash during database migration/initialization.</t>
         </is>
       </c>
     </row>
@@ -1472,17 +1472,17 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>System displays an error message stating the account is pending approval. Login is denied.</t>
+          <t>Test execution aborted. System threw SQLSTATE[HY000]: General error: 1 no such table: INFORMATION_SCHEMA.KEY_COLUMN_USAGE.</t>
         </is>
       </c>
       <c r="H3" s="1" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Fail</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>The application uses MySQL-specific raw schema queries (INFORMATION_SCHEMA) which are incompatible with the automated testing environment (SQLite in-memory DB). Tests crash during database migration/initialization.</t>
         </is>
       </c>
     </row>
@@ -1519,17 +1519,17 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>User is successfully authenticated and redirected to the Dashboard.</t>
+          <t>Test execution aborted. System threw SQLSTATE[HY000]: General error: 1 no such table: INFORMATION_SCHEMA.KEY_COLUMN_USAGE.</t>
         </is>
       </c>
       <c r="H4" s="1" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Fail</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>The application uses MySQL-specific raw schema queries (INFORMATION_SCHEMA) which are incompatible with the automated testing environment (SQLite in-memory DB). Tests crash during database migration/initialization.</t>
         </is>
       </c>
     </row>
@@ -1567,17 +1567,17 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>System sends a PIN to the user's email and redirects to the PIN verification page.</t>
+          <t>Test execution aborted. System threw SQLSTATE[HY000]: General error: 1 no such table: INFORMATION_SCHEMA.KEY_COLUMN_USAGE.</t>
         </is>
       </c>
       <c r="H5" s="1" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Fail</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>The application uses MySQL-specific raw schema queries (INFORMATION_SCHEMA) which are incompatible with the automated testing environment (SQLite in-memory DB). Tests crash during database migration/initialization.</t>
         </is>
       </c>
     </row>
@@ -1615,17 +1615,17 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Password is successfully updated. User can now log in with the new password.</t>
+          <t>Test execution aborted. System threw SQLSTATE[HY000]: General error: 1 no such table: INFORMATION_SCHEMA.KEY_COLUMN_USAGE.</t>
         </is>
       </c>
       <c r="H6" s="1" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Fail</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>The application uses MySQL-specific raw schema queries (INFORMATION_SCHEMA) which are incompatible with the automated testing environment (SQLite in-memory DB). Tests crash during database migration/initialization.</t>
         </is>
       </c>
     </row>

</xml_diff>